<commit_message>
Add latest results of factual error experiment
</commit_message>
<xml_diff>
--- a/data/analysis_results/gpt-4.1_vs_Llama-2-7b-chat-hf/Mistral-7B-Instruct-v0.2/aae/total_votes_file.xlsx
+++ b/data/analysis_results/gpt-4.1_vs_Llama-2-7b-chat-hf/Mistral-7B-Instruct-v0.2/aae/total_votes_file.xlsx
@@ -37,10 +37,10 @@
     <t>total</t>
   </si>
   <si>
-    <t>model1-first</t>
-  </si>
-  <si>
-    <t>model2-first</t>
+    <t>gpt-4.1-first</t>
+  </si>
+  <si>
+    <t>meta-llama/Llama-2-7b-chat-hf-first</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Overwrite main with uv-vllm contents
</commit_message>
<xml_diff>
--- a/data/analysis_results/gpt-4.1_vs_Llama-2-7b-chat-hf/Mistral-7B-Instruct-v0.2/aae/total_votes_file.xlsx
+++ b/data/analysis_results/gpt-4.1_vs_Llama-2-7b-chat-hf/Mistral-7B-Instruct-v0.2/aae/total_votes_file.xlsx
@@ -37,10 +37,10 @@
     <t>total</t>
   </si>
   <si>
-    <t>gpt-4.1-first</t>
-  </si>
-  <si>
-    <t>meta-llama/Llama-2-7b-chat-hf-first</t>
+    <t>model1-first</t>
+  </si>
+  <si>
+    <t>model2-first</t>
   </si>
 </sst>
 </file>

</xml_diff>